<commit_message>
chore: update LeetCode log
</commit_message>
<xml_diff>
--- a/data/leetcode_log.xlsx
+++ b/data/leetcode_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -637,6 +637,25 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>46119</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Minimum Depth of Binary Tree
+Walking Robot Simulation II</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>